<commit_message>
Expand OrgChart: 15 families 49 functions, new salary template, Aon-based level definitions
</commit_message>
<xml_diff>
--- a/static/层级定义.xlsx
+++ b/static/层级定义.xlsx
@@ -74,7 +74,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -451,8 +451,8 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="65" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -487,7 +487,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="60" customHeight="1">
+    <row r="2" ht="100" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Level 1</t>
@@ -510,16 +510,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>入门级岗位。在直接指导下完成基础性、重复性工作，无需独立决策。通常为应届或1年以内工作经验。</t>
+          <t>入门/辅助级岗位。完成已确定工序的日常工作，受直接监督，遵照指示办事。工作内容重复性强，无需独立判断和决策。包括一般行政辅助、流水线操作等基础执行岗位。
+通常为应届或1年以内工作经验。</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>实习生、初级文员</t>
+          <t>前台、文员、行政助理、仓库管理员</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="60" customHeight="1">
+    <row r="3" ht="100" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Level 2</t>
@@ -542,16 +543,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>初级执行岗位。在指导下独立完成单一模块的日常工作，开始积累专业技能。通常1-3年工作经验。</t>
+          <t>初级执行岗位。在指导下独立完成单一模块的日常工作，开始积累专业技能。受主管有限监督，具有在某一专业技术领域或行政职能领域的基础知识。影响力通常局限于直接工作领域。
+通常1-3年工作经验。</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>招聘助理、薪酬助理、培训助理</t>
+          <t>招聘助理、薪酬助理、培训助理、初级工程师</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="60" customHeight="1">
+    <row r="4" ht="100" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Level 3</t>
@@ -574,16 +576,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>独立执行岗位。能够独立完成本专业模块的核心工作，具备扎实的专业基础，可指导初级员工。通常3-5年经验。</t>
+          <t>独立贡献者。不具备人员管理职责，受主管有限监督，具有在某一专业技术领域或行政职能领域广泛的知识和技能。能独立完成本专业模块的核心工作，可指导初级员工。对团队目标实现具有一些间接影响。
+通常3-5年经验。</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>招聘专员、薪酬专员、HRBP专员</t>
+          <t>招聘专员、薪酬专员、HRBP专员、工程师、销售代表、会计</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="60" customHeight="1">
+    <row r="5" ht="100" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Level 4</t>
@@ -606,16 +609,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>资深执行或基层管理岗位。专业通道上是模块内的技术骨干，能处理复杂问题；管理通道上开始带小团队（3-8人），对团队产出负责。通常5-8年经验。</t>
+          <t>资深执行或基层管理岗位。专业通道上是模块内的技术骨干，能处理复杂问题，可能领导小型项目；管理通道上负责某一次级部门或团队的日常管理，监管员工的工作、考核绩效（通常3-8人）。对所在团队/项目的目标实现具有重要影响，对部门或小组的决策产生影响。
+通常5-8年经验。</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>高级招聘专员、招聘主管、HRBP主管</t>
+          <t>高级招聘专员、招聘主管、高级工程师、销售主管、高级金融分析师</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1">
+    <row r="6" ht="100" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Level 5</t>
@@ -638,16 +642,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>专家或中层管理岗位。专业通道上是跨模块的资深专家，能制定专业标准和方法论；管理通道上管理一个完整职能团队（8-20人），对部门目标负责。通常8-12年经验。</t>
+          <t>部门经理或跨模块资深专家。作为第一线的管理人员，管理一个主要部门的活动，制定部门目标、政策、工作程序；或领导对公司目标实现具有重要意义的大型项目。对所负责团队的目标和业绩的实现具有关键影响力，参与部门重要决策的制定。
+通常8-12年经验。</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>招聘经理、薪酬经理、资深HRBP</t>
+          <t>招聘经理、薪酬经理、HRBP经理、生产经理、财务经理、工程部经理</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1">
+    <row r="7" ht="100" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Level 6</t>
@@ -670,16 +675,17 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>高级专家或高层管理岗位。专业通道上是行业级别的专家，能影响公司战略决策；管理通道上管理多个团队或跨部门协调，对业务线目标负责。通常12-18年经验。</t>
+          <t>高级经理或行业级专家。对某一业务部门或主要的职能部门的短期和长期的经营决策起着重要的作用；指导和协调跨部门的活动；制定业务部门或主要职能部门的政策。对业务部门或主要职能部门的目标实现负有重大责任。对公司一主要业务单元/部门或主要职能领域的目标完成和业绩具有关键的影响力。
+通常12-18年经验。</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>招聘专家、高级薪酬经理、OD专家</t>
+          <t>高级招聘经理、招聘专家、薪酬专家、OD专家、副总经理、三级销售经理</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1">
+    <row r="8" ht="100" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Level 7</t>
@@ -702,12 +708,13 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>高管或总监级岗位。对整个职能领域的战略方向和业务结果负最终责任，参与公司核心管理决策，管理大型团队或多个部门。通常15年以上经验。</t>
+          <t>总监或公司级高管。某一国家设立的公司的最高负责人，制定和诠释公司层面的政策，组织公司层面的跨业务部门的项目，影响公司的总体发展方向。对公司的目标实现负有重大责任，参与公司战略决策和公司整体经营目标的制定。调配公司某一方面的重要资源（市场、财务或人力资源等）。
+通常15年以上经验。</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>招聘总监、HRBP总监、OD总监</t>
+          <t>招聘总监、HRBP总监、OD总监、总经理、总裁、厂长</t>
         </is>
       </c>
     </row>

</xml_diff>